<commit_message>
feat(guests): Open in Google Sheets; import skips a how-to line above the headings
Templates move the how-to to its own sheet; generic how-to drops Side.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/web/public/templates/setnayan-guest-list-wedding.xlsx
+++ b/apps/web/public/templates/setnayan-guest-list-wedding.xlsx
@@ -4,11 +4,12 @@
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guests" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="2" state="hidden" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guests" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" state="hidden" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -36,6 +37,10 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="14"/>
     </font>
   </fonts>
   <fills count="3">
@@ -63,13 +68,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -435,7 +444,38 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:A3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="90" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>How to fill in this guest list</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="90" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>One guest per row. Only First name and Last name are needed. Pick Side, Group and Role from the little arrows. Their guests (+) = how many people they may bring. Save, then upload it in Setnayan (Guests › + › Import from a file).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -450,211 +490,194 @@
     <col width="18" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>One guest per row. Only First name and Last name are needed. Pick Side, Group and Role from the little arrows. Their guests (+) = how many people they may bring. Save, then upload it in Setnayan (Guests › + › Import from a file).</t>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Prefix</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>First name</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Middle name</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Last name</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Suffix</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Side</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Their guests (+)</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Mobile (optional)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Prefix</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>First name</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Middle name</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Last name</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Suffix</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Side</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Group</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Role</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>Their guests (+)</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>Mobile (optional)</t>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Mr.</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Manuel</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Cortez</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Casasola</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Groom</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Principal Sponsor (Ninong)</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Mr.</t>
+          <t>Ms.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Manuel</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Cortez</t>
+          <t>Maria</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Casasola</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr"/>
+          <t>Santos</t>
+        </is>
+      </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Groom</t>
+          <t>Bride</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Family</t>
+          <t>Friends</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Principal Sponsor (Ninong)</t>
+          <t>Bridesmaid</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>+63 917 123 4567</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Juan</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Reyes</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Jr.</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Work</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Guest</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Ms.</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Maria</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Santos</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Bride</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Friends</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Bridesmaid</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>+63 917 123 4567</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr"/>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Juan</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Reyes</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Jr.</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Work</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Guest</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:J1"/>
-  </mergeCells>
   <dataValidations count="5">
-    <dataValidation sqref="A3:A1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick from the list" type="list">
+    <dataValidation sqref="A2:A1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick from the list" type="list">
       <formula1>=Lists!$A$2:$A$10</formula1>
     </dataValidation>
-    <dataValidation sqref="F3:F1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick from the list" type="list">
+    <dataValidation sqref="F2:F1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick from the list" type="list">
       <formula1>=Lists!$B$2:$B$4</formula1>
     </dataValidation>
-    <dataValidation sqref="G3:G1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick from the list" type="list">
+    <dataValidation sqref="G2:G1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick from the list" type="list">
       <formula1>=Lists!$C$2:$C$6</formula1>
     </dataValidation>
-    <dataValidation sqref="H3:H1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick from the list" type="list">
+    <dataValidation sqref="H2:H1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick from the list" type="list">
       <formula1>=Lists!$D$2:$D$25</formula1>
     </dataValidation>
-    <dataValidation sqref="I3:I1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick from the list" type="list">
+    <dataValidation sqref="I2:I1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick from the list" type="list">
       <formula1>=Lists!$E$2:$E$6</formula1>
     </dataValidation>
   </dataValidations>
@@ -662,7 +685,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>